<commit_message>
Upgraded the  system...fixed the bugs...still beta version
</commit_message>
<xml_diff>
--- a/data/Master.xlsx
+++ b/data/Master.xlsx
@@ -12,10 +12,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Processing_Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review_Required" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Trace" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File_Breakdown" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cleaned_Master'!$A$1:$K$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Source_Trace'!$A$1:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cleaned_Master'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Source_Trace'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'File_Breakdown'!$A$1:$F$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -49,7 +51,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -86,6 +88,12 @@
         <bgColor rgb="00595959"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00333333"/>
+        <bgColor rgb="00333333"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -113,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -136,6 +144,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -502,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -510,12 +521,9 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="41" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -546,30 +554,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Business Name</t>
+          <t>Annual Revenue</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Contact Number</t>
+          <t>Website</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Email Address</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Annual Revenue</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Website</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -601,12 +594,13 @@
           <t>60601</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>$1200000</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -637,9 +631,6 @@
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -670,9 +661,6 @@
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -701,15 +689,12 @@
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>https://stark.com</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Key defense partner; priority account</t>
         </is>
@@ -744,210 +729,159 @@
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Wayne Technologies</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>555-0600</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>bruce@wayne.com</t>
+        </is>
+      </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Gotham</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Acme Industrial</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>555-0100</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>contact@acme.com</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>$1200000</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+          <t>$50000000</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Globex Corp.</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>555-0200</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>info@globex.com</t>
+        </is>
+      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Gotham</t>
+          <t>Springfield</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Wayne Technologies</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>555-0600</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>bruce@wayne.com</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>$50000000</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
+          <t>$8500000</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Cyberdyne Systems</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>555-0700</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>miles@cyberdyne.com</t>
+        </is>
+      </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Springfield</t>
+          <t>Sunnyvale</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Globex Corp.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>555-0200</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>info@globex.com</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>$8500000</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
+          <t>$25000000</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Sunnyvale</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Soylent Food Corp</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>555-0800</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>orders@soylent.com</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Cyberdyne Systems</t>
-        </is>
-      </c>
+      <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>555-0700</t>
+          <t>https://soylent.com</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>miles@cyberdyne.com</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>$25000000</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+          <t>Consumer goods</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Soylent Food Corp</t>
+          <t>Massive Dynamic</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>555-0800</t>
+          <t>555-0900</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>orders@soylent.com</t>
+          <t>inquiry@massivedynamic.com</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
-      <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>https://soylent.com</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
-          <t>Consumer goods</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Massive Dynamic</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>555-0900</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>inquiry@massivedynamic.com</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>https://massivedynamic.com</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R&amp;D lab</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K12"/>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1111,7 +1045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1119,6 +1053,7 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1147,6 +1082,11 @@
           <t>_import_id</t>
         </is>
       </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>_is_master</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="8" t="n">
@@ -1167,8 +1107,11 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>companies_batch1.xlsx_20261027_175107</t>
-        </is>
+          <t>companies_batch1.xlsx_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
@@ -1190,8 +1133,11 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>companies_batch1.xlsx_20261027_175107</t>
-        </is>
+          <t>companies_batch1.xlsx_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
@@ -1213,8 +1159,11 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>companies_batch1.xlsx_20261027_175107</t>
-        </is>
+          <t>companies_batch1.xlsx_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -1236,8 +1185,11 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>companies_batch1.xlsx_20261027_175107</t>
-        </is>
+          <t>companies_batch1.xlsx_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -1259,8 +1211,11 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>companies_batch1.xlsx_20261027_175107</t>
-        </is>
+          <t>companies_batch1.xlsx_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -1278,12 +1233,15 @@
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>customers.csv_20261027_175107</t>
-        </is>
+          <t>customers.csv_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -1301,12 +1259,15 @@
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>customers.csv_20261027_175107</t>
-        </is>
+          <t>customers.csv_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -1324,12 +1285,15 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>customers.csv_20261027_175107</t>
-        </is>
+          <t>customers.csv_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -1338,7 +1302,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>customers.csv</t>
+          <t>partners_semicolon.csv</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1347,12 +1311,15 @@
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>customers.csv_20261027_175107</t>
-        </is>
+          <t>partners_semicolon.csv_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -1370,39 +1337,178 @@
         </is>
       </c>
       <c r="D11" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>partners_semicolon.csv_20261028_092550</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Filename</t>
+        </is>
+      </c>
+      <c r="B1" s="9" t="inlineStr">
+        <is>
+          <t>Worksheet</t>
+        </is>
+      </c>
+      <c r="C1" s="9" t="inlineStr">
+        <is>
+          <t>Rows Read</t>
+        </is>
+      </c>
+      <c r="D1" s="9" t="inlineStr">
+        <is>
+          <t>New Records Contributed</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Duplicates Excluded</t>
+        </is>
+      </c>
+      <c r="F1" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>companies_batch1.xlsx</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Active_Companies</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>companies_batch1.xlsx</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Pending_Companies</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>partners_semicolon.csv_20261027_175107</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="8" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="D3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>customers.csv</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CSV_Data</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>partners_semicolon.csv</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>CSV_Data</t>
         </is>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="C5" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>partners_semicolon.csv_20261027_175107</t>
+      <c r="D5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Success</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:F5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>